<commit_message>
feat: cấu hình ngưỡng cảnh báo tồn kho, cọc vỏ nhập tay, xuất điều phối thêm SĐT/Chỉ tiêu
- Cấu hình chung: thêm "Ngưỡng cảnh báo tồn kho" (mặc định 20) — dùng thống nhất ở màn
  Tồn kho, Bảng điều khiển, cảnh báo/chuông (thay ngưỡng cứng theo từng dòng).
- Đơn hàng: thêm ô "Tiền cọc vỏ" cho người dùng tự điền, để trống thì tự tính
  (số bình × phí cọc); thêm cột orders.deposit_override + migration cho CSDL cũ.
- Đơn hàng: bỏ trường "Ghi chú đơn hàng", đưa "Ghi chú giao" lên khối thông tin đơn.
- Xuất Excel điều phối: thêm cột "Số điện thoại" (sau khách hàng) và "Chỉ tiêu" (sau kho).
- migrate T10: sinh revenue_transactions cho đơn đã thu tiền để khớp sổ quỹ.

Co-authored-by: CommandCodeBot <noreply@commandcode.ai>
</commit_message>
<xml_diff>
--- a/excel/qaromi-nhap-T10.xlsx
+++ b/excel/qaromi-nhap-T10.xlsx
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3351" uniqueCount="1322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3459" uniqueCount="1359">
   <si>
     <t>id</t>
   </si>
@@ -123,7 +123,7 @@
     <t>Giám đốc</t>
   </si>
   <si>
-    <t>2026-10-06 14:01:39</t>
+    <t>2026-10-06 14:16:45</t>
   </si>
   <si>
     <t>NV002</t>
@@ -3439,6 +3439,117 @@
   </si>
   <si>
     <t>collected_by</t>
+  </si>
+  <si>
+    <t>PT-20260929-001</t>
+  </si>
+  <si>
+    <t>WATER_SALE</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 8)</t>
+  </si>
+  <si>
+    <t>PT-20260930-001</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 14)</t>
+  </si>
+  <si>
+    <t>PT-20260930-002</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 16)</t>
+  </si>
+  <si>
+    <t>PT-20261001-001</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 24)</t>
+  </si>
+  <si>
+    <t>PT-20261001-002</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 31)</t>
+  </si>
+  <si>
+    <t>PT-20261001-003</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 34)</t>
+  </si>
+  <si>
+    <t>PT-20261001-004</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 35)</t>
+  </si>
+  <si>
+    <t>PT-20261002-001</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 36)</t>
+  </si>
+  <si>
+    <t>PT-20261002-002</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 47)</t>
+  </si>
+  <si>
+    <t>PT-20261002-003</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 50)</t>
+  </si>
+  <si>
+    <t>PT-20261003-001</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 56)</t>
+  </si>
+  <si>
+    <t>PT-20261003-002</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 61)</t>
+  </si>
+  <si>
+    <t>PT-20261003-003</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 64)</t>
+  </si>
+  <si>
+    <t>PT-20261005-001</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 68)</t>
+  </si>
+  <si>
+    <t>PT-20261005-002</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 76)</t>
+  </si>
+  <si>
+    <t>PT-20261005-003</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 77)</t>
+  </si>
+  <si>
+    <t>PT-20261005-004</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 83)</t>
+  </si>
+  <si>
+    <t>PT-20261005-005</t>
+  </si>
+  <si>
+    <t>Thu tiền đơn nhập từ sổ ĐIỀU PHỐI NƯỚC LỌC T10 (dòng 87)</t>
   </si>
   <si>
     <t>expense_code</t>
@@ -13441,7 +13552,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -13477,6 +13588,636 @@
       </c>
       <c r="K1" s="1" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1129</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>3</v>
+      </c>
+      <c r="F2">
+        <v>980000</v>
+      </c>
+      <c r="G2" t="s">
+        <v>822</v>
+      </c>
+      <c r="H2">
+        <v>195</v>
+      </c>
+      <c r="I2" t="s">
+        <v>704</v>
+      </c>
+      <c r="J2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="K2" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D3">
+        <v>9</v>
+      </c>
+      <c r="E3">
+        <v>7</v>
+      </c>
+      <c r="F3">
+        <v>490000</v>
+      </c>
+      <c r="G3" t="s">
+        <v>822</v>
+      </c>
+      <c r="H3">
+        <v>195</v>
+      </c>
+      <c r="I3" t="s">
+        <v>834</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1133</v>
+      </c>
+      <c r="K3" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D4">
+        <v>11</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>255000</v>
+      </c>
+      <c r="G4" t="s">
+        <v>812</v>
+      </c>
+      <c r="H4">
+        <v>51</v>
+      </c>
+      <c r="I4" t="s">
+        <v>834</v>
+      </c>
+      <c r="J4" t="s">
+        <v>1135</v>
+      </c>
+      <c r="K4" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1136</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D5">
+        <v>19</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>490000</v>
+      </c>
+      <c r="G5" t="s">
+        <v>822</v>
+      </c>
+      <c r="H5">
+        <v>196</v>
+      </c>
+      <c r="I5" t="s">
+        <v>701</v>
+      </c>
+      <c r="J5" t="s">
+        <v>1137</v>
+      </c>
+      <c r="K5" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D6">
+        <v>25</v>
+      </c>
+      <c r="E6">
+        <v>14</v>
+      </c>
+      <c r="F6">
+        <v>260000</v>
+      </c>
+      <c r="G6" t="s">
+        <v>822</v>
+      </c>
+      <c r="H6">
+        <v>195</v>
+      </c>
+      <c r="I6" t="s">
+        <v>701</v>
+      </c>
+      <c r="J6" t="s">
+        <v>1139</v>
+      </c>
+      <c r="K6" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1140</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D7">
+        <v>28</v>
+      </c>
+      <c r="E7">
+        <v>16</v>
+      </c>
+      <c r="F7">
+        <v>52000</v>
+      </c>
+      <c r="G7" t="s">
+        <v>812</v>
+      </c>
+      <c r="H7">
+        <v>38</v>
+      </c>
+      <c r="I7" t="s">
+        <v>701</v>
+      </c>
+      <c r="J7" t="s">
+        <v>1141</v>
+      </c>
+      <c r="K7" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1142</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D8">
+        <v>29</v>
+      </c>
+      <c r="E8">
+        <v>17</v>
+      </c>
+      <c r="F8">
+        <v>510000</v>
+      </c>
+      <c r="G8" t="s">
+        <v>822</v>
+      </c>
+      <c r="H8">
+        <v>51</v>
+      </c>
+      <c r="I8" t="s">
+        <v>701</v>
+      </c>
+      <c r="J8" t="s">
+        <v>1143</v>
+      </c>
+      <c r="K8" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1144</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D9">
+        <v>30</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9">
+        <v>1150000</v>
+      </c>
+      <c r="G9" t="s">
+        <v>822</v>
+      </c>
+      <c r="H9">
+        <v>4</v>
+      </c>
+      <c r="I9" t="s">
+        <v>921</v>
+      </c>
+      <c r="J9" t="s">
+        <v>1145</v>
+      </c>
+      <c r="K9" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1146</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D10">
+        <v>40</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10">
+        <v>980000</v>
+      </c>
+      <c r="G10" t="s">
+        <v>822</v>
+      </c>
+      <c r="H10">
+        <v>4</v>
+      </c>
+      <c r="I10" t="s">
+        <v>921</v>
+      </c>
+      <c r="J10" t="s">
+        <v>1147</v>
+      </c>
+      <c r="K10" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1148</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D11">
+        <v>43</v>
+      </c>
+      <c r="E11">
+        <v>20</v>
+      </c>
+      <c r="F11">
+        <v>52000</v>
+      </c>
+      <c r="G11" t="s">
+        <v>822</v>
+      </c>
+      <c r="H11">
+        <v>14</v>
+      </c>
+      <c r="I11" t="s">
+        <v>921</v>
+      </c>
+      <c r="J11" t="s">
+        <v>1149</v>
+      </c>
+      <c r="K11" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1150</v>
+      </c>
+      <c r="C12" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D12">
+        <v>49</v>
+      </c>
+      <c r="E12">
+        <v>17</v>
+      </c>
+      <c r="F12">
+        <v>170000</v>
+      </c>
+      <c r="G12" t="s">
+        <v>822</v>
+      </c>
+      <c r="H12">
+        <v>14</v>
+      </c>
+      <c r="I12" t="s">
+        <v>702</v>
+      </c>
+      <c r="J12" t="s">
+        <v>1151</v>
+      </c>
+      <c r="K12" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C13" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D13">
+        <v>54</v>
+      </c>
+      <c r="E13">
+        <v>26</v>
+      </c>
+      <c r="F13">
+        <v>144000</v>
+      </c>
+      <c r="G13" t="s">
+        <v>822</v>
+      </c>
+      <c r="H13">
+        <v>4</v>
+      </c>
+      <c r="I13" t="s">
+        <v>702</v>
+      </c>
+      <c r="J13" t="s">
+        <v>1153</v>
+      </c>
+      <c r="K13" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1154</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D14">
+        <v>57</v>
+      </c>
+      <c r="E14">
+        <v>28</v>
+      </c>
+      <c r="F14">
+        <v>490000</v>
+      </c>
+      <c r="G14" t="s">
+        <v>822</v>
+      </c>
+      <c r="H14">
+        <v>86</v>
+      </c>
+      <c r="I14" t="s">
+        <v>702</v>
+      </c>
+      <c r="J14" t="s">
+        <v>1155</v>
+      </c>
+      <c r="K14" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1156</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D15">
+        <v>61</v>
+      </c>
+      <c r="E15">
+        <v>26</v>
+      </c>
+      <c r="F15">
+        <v>48000</v>
+      </c>
+      <c r="G15" t="s">
+        <v>822</v>
+      </c>
+      <c r="H15">
+        <v>195</v>
+      </c>
+      <c r="I15" t="s">
+        <v>700</v>
+      </c>
+      <c r="J15" t="s">
+        <v>1157</v>
+      </c>
+      <c r="K15" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1158</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D16">
+        <v>68</v>
+      </c>
+      <c r="E16">
+        <v>2</v>
+      </c>
+      <c r="F16">
+        <v>980000</v>
+      </c>
+      <c r="G16" t="s">
+        <v>822</v>
+      </c>
+      <c r="H16">
+        <v>195</v>
+      </c>
+      <c r="I16" t="s">
+        <v>700</v>
+      </c>
+      <c r="J16" t="s">
+        <v>1159</v>
+      </c>
+      <c r="K16" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1160</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D17">
+        <v>69</v>
+      </c>
+      <c r="E17">
+        <v>26</v>
+      </c>
+      <c r="F17">
+        <v>980000</v>
+      </c>
+      <c r="G17" t="s">
+        <v>822</v>
+      </c>
+      <c r="H17">
+        <v>196</v>
+      </c>
+      <c r="I17" t="s">
+        <v>700</v>
+      </c>
+      <c r="J17" t="s">
+        <v>1161</v>
+      </c>
+      <c r="K17" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1162</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D18">
+        <v>74</v>
+      </c>
+      <c r="E18">
+        <v>36</v>
+      </c>
+      <c r="F18">
+        <v>294000</v>
+      </c>
+      <c r="G18" t="s">
+        <v>822</v>
+      </c>
+      <c r="H18">
+        <v>20</v>
+      </c>
+      <c r="I18" t="s">
+        <v>700</v>
+      </c>
+      <c r="J18" t="s">
+        <v>1163</v>
+      </c>
+      <c r="K18" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D19">
+        <v>78</v>
+      </c>
+      <c r="E19">
+        <v>28</v>
+      </c>
+      <c r="F19">
+        <v>294000</v>
+      </c>
+      <c r="G19" t="s">
+        <v>822</v>
+      </c>
+      <c r="H19">
+        <v>86</v>
+      </c>
+      <c r="I19" t="s">
+        <v>700</v>
+      </c>
+      <c r="J19" t="s">
+        <v>1165</v>
+      </c>
+      <c r="K19" t="s">
+        <v>743</v>
       </c>
     </row>
   </sheetData>
@@ -13495,19 +14236,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1129</v>
+        <v>1166</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1130</v>
+        <v>1167</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1127</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1131</v>
+        <v>1168</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1132</v>
+        <v>1169</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
@@ -13516,7 +14257,7 @@
         <v>779</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>1133</v>
+        <v>1170</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>713</v>
@@ -13547,13 +14288,13 @@
         <v>477</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1134</v>
+        <v>1171</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1106</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1135</v>
+        <v>1172</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>19</v>
@@ -13587,7 +14328,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1136</v>
+        <v>1173</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>19</v>
@@ -13604,10 +14345,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>1137</v>
+        <v>1174</v>
       </c>
       <c r="C2" t="s">
-        <v>1138</v>
+        <v>1175</v>
       </c>
       <c r="D2">
         <v>5000</v>
@@ -13616,7 +14357,7 @@
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>1139</v>
+        <v>1176</v>
       </c>
     </row>
   </sheetData>
@@ -13647,19 +14388,19 @@
         <v>477</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1140</v>
+        <v>1177</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1141</v>
+        <v>1178</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>1142</v>
+        <v>1179</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>1143</v>
+        <v>1180</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>1144</v>
+        <v>1181</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>19</v>
@@ -17849,13 +18590,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1145</v>
+        <v>1182</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1146</v>
+        <v>1183</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1147</v>
+        <v>1184</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1105</v>
@@ -17864,13 +18605,13 @@
         <v>769</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1148</v>
+        <v>1185</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>1149</v>
+        <v>1186</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>1150</v>
+        <v>1187</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>526</v>
@@ -17888,7 +18629,7 @@
         <v>781</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>1151</v>
+        <v>1188</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>788</v>
@@ -17900,7 +18641,7 @@
         <v>792</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>1152</v>
+        <v>1189</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>713</v>
@@ -17977,16 +18718,16 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1153</v>
+        <v>1190</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1154</v>
+        <v>1191</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>662</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1155</v>
+        <v>1192</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>19</v>
@@ -18000,13 +18741,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>1156</v>
+        <v>1193</v>
       </c>
       <c r="C2" t="s">
-        <v>1157</v>
+        <v>1194</v>
       </c>
       <c r="E2" t="s">
-        <v>1158</v>
+        <v>1195</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -18015,7 +18756,7 @@
         <v>1</v>
       </c>
       <c r="I2" t="s">
-        <v>1159</v>
+        <v>1196</v>
       </c>
     </row>
   </sheetData>
@@ -18054,16 +18795,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>1160</v>
+        <v>1197</v>
       </c>
       <c r="C2" t="s">
-        <v>1161</v>
+        <v>1198</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>1139</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -18071,16 +18812,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>1162</v>
+        <v>1199</v>
       </c>
       <c r="C3" t="s">
-        <v>1163</v>
+        <v>1200</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>1139</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -18088,16 +18829,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>1164</v>
+        <v>1201</v>
       </c>
       <c r="C4" t="s">
-        <v>1165</v>
+        <v>1202</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>1139</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -18105,7 +18846,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>1166</v>
+        <v>1203</v>
       </c>
       <c r="C5" t="s">
         <v>154</v>
@@ -18114,7 +18855,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>1139</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -18122,7 +18863,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>1167</v>
+        <v>1204</v>
       </c>
       <c r="C6" t="s">
         <v>157</v>
@@ -18131,7 +18872,7 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>1139</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -18139,7 +18880,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>1168</v>
+        <v>1205</v>
       </c>
       <c r="C7" t="s">
         <v>355</v>
@@ -18148,7 +18889,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>1139</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -18156,7 +18897,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>1169</v>
+        <v>1206</v>
       </c>
       <c r="C8" t="s">
         <v>358</v>
@@ -18165,7 +18906,7 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>1139</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -18173,16 +18914,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>1170</v>
+        <v>1207</v>
       </c>
       <c r="C9" t="s">
-        <v>1171</v>
+        <v>1208</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>1139</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -18190,16 +18931,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>1172</v>
+        <v>1209</v>
       </c>
       <c r="C10" t="s">
-        <v>1173</v>
+        <v>1210</v>
       </c>
       <c r="E10">
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>1139</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -18207,16 +18948,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>1174</v>
+        <v>1211</v>
       </c>
       <c r="C11" t="s">
-        <v>1175</v>
+        <v>1212</v>
       </c>
       <c r="E11">
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>1139</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -18224,16 +18965,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>1213</v>
+      </c>
+      <c r="C12" t="s">
+        <v>1214</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
         <v>1176</v>
-      </c>
-      <c r="C12" t="s">
-        <v>1177</v>
-      </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
-      <c r="F12" t="s">
-        <v>1139</v>
       </c>
     </row>
   </sheetData>
@@ -18272,10 +19013,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>1178</v>
+        <v>1215</v>
       </c>
       <c r="C2" t="s">
-        <v>1179</v>
+        <v>1216</v>
       </c>
       <c r="D2" t="s">
         <v>452</v>
@@ -18284,7 +19025,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>1159</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -18292,10 +19033,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>1180</v>
+        <v>1217</v>
       </c>
       <c r="C3" t="s">
-        <v>1181</v>
+        <v>1218</v>
       </c>
       <c r="D3" t="s">
         <v>452</v>
@@ -18304,7 +19045,7 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>1159</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -18312,10 +19053,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>1182</v>
+        <v>1219</v>
       </c>
       <c r="C4" t="s">
-        <v>1183</v>
+        <v>1220</v>
       </c>
       <c r="D4" t="s">
         <v>452</v>
@@ -18324,7 +19065,7 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>1159</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -18332,10 +19073,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>1184</v>
+        <v>1221</v>
       </c>
       <c r="C5" t="s">
-        <v>1185</v>
+        <v>1222</v>
       </c>
       <c r="D5" t="s">
         <v>452</v>
@@ -18344,7 +19085,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>1159</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -18352,13 +19093,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>1186</v>
+        <v>1223</v>
       </c>
       <c r="C6" t="s">
-        <v>1187</v>
+        <v>1224</v>
       </c>
       <c r="D6" t="s">
-        <v>1188</v>
+        <v>1225</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -18412,28 +19153,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>1189</v>
+        <v>1226</v>
       </c>
       <c r="C2" t="s">
-        <v>1190</v>
+        <v>1227</v>
       </c>
       <c r="D2" t="s">
-        <v>1191</v>
+        <v>1228</v>
       </c>
       <c r="E2" t="s">
-        <v>1192</v>
+        <v>1229</v>
       </c>
       <c r="F2" t="s">
-        <v>1193</v>
+        <v>1230</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>1194</v>
+        <v>1231</v>
       </c>
       <c r="I2" t="s">
-        <v>1159</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -18441,28 +19182,28 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>1195</v>
+        <v>1232</v>
       </c>
       <c r="C3" t="s">
+        <v>1233</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1234</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1235</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1236</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1231</v>
+      </c>
+      <c r="I3" t="s">
         <v>1196</v>
-      </c>
-      <c r="D3" t="s">
-        <v>1197</v>
-      </c>
-      <c r="E3" t="s">
-        <v>1198</v>
-      </c>
-      <c r="F3" t="s">
-        <v>1199</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3" t="s">
-        <v>1194</v>
-      </c>
-      <c r="I3" t="s">
-        <v>1159</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -18470,16 +19211,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>1200</v>
+        <v>1237</v>
       </c>
       <c r="C4" t="s">
-        <v>1201</v>
+        <v>1238</v>
       </c>
       <c r="G4">
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>1202</v>
+        <v>1239</v>
       </c>
       <c r="I4" t="s">
         <v>23</v>
@@ -18490,16 +19231,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>1203</v>
+        <v>1240</v>
       </c>
       <c r="C5" t="s">
-        <v>1204</v>
+        <v>1241</v>
       </c>
       <c r="G5">
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>1202</v>
+        <v>1239</v>
       </c>
       <c r="I5" t="s">
         <v>23</v>
@@ -18510,16 +19251,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>1205</v>
+        <v>1242</v>
       </c>
       <c r="C6" t="s">
-        <v>1206</v>
+        <v>1243</v>
       </c>
       <c r="G6">
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>1202</v>
+        <v>1239</v>
       </c>
       <c r="I6" t="s">
         <v>23</v>
@@ -18530,16 +19271,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>1207</v>
+        <v>1244</v>
       </c>
       <c r="C7" t="s">
-        <v>1208</v>
+        <v>1245</v>
       </c>
       <c r="G7">
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>1202</v>
+        <v>1239</v>
       </c>
       <c r="I7" t="s">
         <v>23</v>
@@ -18550,16 +19291,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>1209</v>
+        <v>1246</v>
       </c>
       <c r="C8" t="s">
-        <v>1210</v>
+        <v>1247</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>1202</v>
+        <v>1239</v>
       </c>
       <c r="I8" t="s">
         <v>23</v>
@@ -18581,10 +19322,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1211</v>
+        <v>1248</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1212</v>
+        <v>1249</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1108</v>
@@ -18593,7 +19334,7 @@
         <v>7</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1213</v>
+        <v>1250</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>713</v>
@@ -18621,10 +19362,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1214</v>
+        <v>1251</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1215</v>
+        <v>1252</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>694</v>
@@ -18642,28 +19383,28 @@
         <v>1105</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>1216</v>
+        <v>1253</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>1113</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>1217</v>
+        <v>1254</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>1218</v>
+        <v>1255</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>1219</v>
+        <v>1256</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>713</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>1220</v>
+        <v>1257</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>1221</v>
+        <v>1258</v>
       </c>
       <c r="R1" s="1" t="s">
         <v>5</v>
@@ -18691,7 +19432,7 @@
         <v>695</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1222</v>
+        <v>1259</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>696</v>
@@ -18700,7 +19441,7 @@
         <v>709</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1223</v>
+        <v>1260</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>713</v>
@@ -18722,16 +19463,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1224</v>
+        <v>1261</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1225</v>
+        <v>1262</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1226</v>
+        <v>1263</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1227</v>
+        <v>1264</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
@@ -18826,13 +19567,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1228</v>
+        <v>1265</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1229</v>
+        <v>1266</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1230</v>
+        <v>1267</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>713</v>
@@ -18846,22 +19587,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>1231</v>
+        <v>1268</v>
       </c>
       <c r="C2" t="s">
-        <v>1232</v>
+        <v>1269</v>
       </c>
       <c r="D2">
         <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>1233</v>
+        <v>1270</v>
       </c>
       <c r="G2" t="s">
-        <v>1234</v>
+        <v>1271</v>
       </c>
       <c r="H2" t="s">
-        <v>1139</v>
+        <v>1176</v>
       </c>
     </row>
   </sheetData>
@@ -18883,7 +19624,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1235</v>
+        <v>1272</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>769</v>
@@ -18920,10 +19661,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>1236</v>
+        <v>1273</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1237</v>
+        <v>1274</v>
       </c>
     </row>
   </sheetData>
@@ -18942,37 +19683,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1238</v>
+        <v>1275</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1239</v>
+        <v>1276</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1240</v>
+        <v>1277</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1241</v>
+        <v>1278</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1242</v>
+        <v>1279</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1243</v>
+        <v>1280</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>1244</v>
+        <v>1281</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>1245</v>
+        <v>1282</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>1246</v>
+        <v>1283</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>1247</v>
+        <v>1284</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>1248</v>
+        <v>1285</v>
       </c>
     </row>
   </sheetData>
@@ -18994,10 +19735,10 @@
         <v>1105</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1249</v>
+        <v>1286</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1250</v>
+        <v>1287</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>694</v>
@@ -19006,7 +19747,7 @@
         <v>711</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1251</v>
+        <v>1288</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>1127</v>
@@ -19034,7 +19775,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1252</v>
+        <v>1289</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>695</v>
@@ -19062,37 +19803,37 @@
         <v>1105</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1253</v>
+        <v>1290</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>711</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1254</v>
+        <v>1291</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1255</v>
+        <v>1292</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1256</v>
+        <v>1293</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>1257</v>
+        <v>1294</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>1258</v>
+        <v>1295</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>1259</v>
+        <v>1296</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>1260</v>
+        <v>1297</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>1261</v>
+        <v>1298</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>1262</v>
+        <v>1299</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>713</v>
@@ -19137,7 +19878,7 @@
         <v>50000</v>
       </c>
       <c r="D2" t="s">
-        <v>1263</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -19151,7 +19892,7 @@
         <v>50000</v>
       </c>
       <c r="D3" t="s">
-        <v>1264</v>
+        <v>1301</v>
       </c>
     </row>
   </sheetData>
@@ -19805,57 +20546,57 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>1265</v>
+        <v>1302</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1266</v>
+        <v>1303</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1267</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1268</v>
+        <v>1305</v>
       </c>
       <c r="B2" t="s">
         <v>701</v>
       </c>
       <c r="C2" t="s">
-        <v>1269</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1270</v>
+        <v>1307</v>
       </c>
       <c r="B3" t="s">
-        <v>1271</v>
+        <v>1308</v>
       </c>
       <c r="C3" t="s">
-        <v>1269</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1272</v>
+        <v>1309</v>
       </c>
       <c r="B4" t="s">
-        <v>1273</v>
+        <v>1310</v>
       </c>
       <c r="C4" t="s">
-        <v>1159</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1274</v>
+        <v>1311</v>
       </c>
       <c r="B5" t="s">
-        <v>1273</v>
+        <v>1310</v>
       </c>
       <c r="C5" t="s">
-        <v>1159</v>
+        <v>1196</v>
       </c>
     </row>
   </sheetData>
@@ -19876,18 +20617,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>1275</v>
+        <v>1312</v>
       </c>
       <c r="B1" t="s">
-        <v>1276</v>
+        <v>1313</v>
       </c>
       <c r="C1" t="s">
-        <v>1277</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1278</v>
+        <v>1315</v>
       </c>
       <c r="B2" t="s">
         <v>452</v>
@@ -19898,10 +20639,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1279</v>
+        <v>1316</v>
       </c>
       <c r="B3" t="s">
-        <v>1280</v>
+        <v>1317</v>
       </c>
       <c r="C3" t="s">
         <v>452</v>
@@ -19909,10 +20650,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1281</v>
+        <v>1318</v>
       </c>
       <c r="B4" t="s">
-        <v>1282</v>
+        <v>1319</v>
       </c>
       <c r="C4" t="s">
         <v>452</v>
@@ -19920,10 +20661,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1283</v>
+        <v>1320</v>
       </c>
       <c r="B5" t="s">
-        <v>1284</v>
+        <v>1321</v>
       </c>
       <c r="C5" t="s">
         <v>452</v>
@@ -19931,10 +20672,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>1285</v>
+        <v>1322</v>
       </c>
       <c r="B6" t="s">
-        <v>1286</v>
+        <v>1323</v>
       </c>
       <c r="C6" t="s">
         <v>452</v>
@@ -19942,10 +20683,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>1287</v>
+        <v>1324</v>
       </c>
       <c r="B7" t="s">
-        <v>1288</v>
+        <v>1325</v>
       </c>
       <c r="C7" t="s">
         <v>452</v>
@@ -19953,10 +20694,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>1289</v>
+        <v>1326</v>
       </c>
       <c r="B8" t="s">
-        <v>1290</v>
+        <v>1327</v>
       </c>
       <c r="C8" t="s">
         <v>452</v>
@@ -19964,10 +20705,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>1291</v>
+        <v>1328</v>
       </c>
       <c r="B9" t="s">
-        <v>1292</v>
+        <v>1329</v>
       </c>
       <c r="C9" t="s">
         <v>452</v>
@@ -19975,10 +20716,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>1293</v>
+        <v>1330</v>
       </c>
       <c r="B10" t="s">
-        <v>1294</v>
+        <v>1331</v>
       </c>
       <c r="C10" t="s">
         <v>452</v>
@@ -19986,10 +20727,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>1295</v>
+        <v>1332</v>
       </c>
       <c r="B11" t="s">
-        <v>1296</v>
+        <v>1333</v>
       </c>
       <c r="C11" t="s">
         <v>452</v>
@@ -19997,10 +20738,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>1297</v>
+        <v>1334</v>
       </c>
       <c r="B12" t="s">
-        <v>1286</v>
+        <v>1323</v>
       </c>
       <c r="C12" t="s">
         <v>452</v>
@@ -20019,7 +20760,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>1298</v>
+        <v>1335</v>
       </c>
       <c r="B14" t="s">
         <v>452</v>
@@ -20033,7 +20774,7 @@
         <v>452</v>
       </c>
       <c r="B15" t="s">
-        <v>1299</v>
+        <v>1336</v>
       </c>
       <c r="C15" t="s">
         <v>452</v>
@@ -20044,7 +20785,7 @@
         <v>452</v>
       </c>
       <c r="B16" t="s">
-        <v>1300</v>
+        <v>1337</v>
       </c>
       <c r="C16" t="s">
         <v>452</v>
@@ -20055,7 +20796,7 @@
         <v>452</v>
       </c>
       <c r="B17" t="s">
-        <v>1301</v>
+        <v>1338</v>
       </c>
       <c r="C17" t="s">
         <v>452</v>
@@ -20066,7 +20807,7 @@
         <v>452</v>
       </c>
       <c r="B18" t="s">
-        <v>1302</v>
+        <v>1339</v>
       </c>
       <c r="C18" t="s">
         <v>452</v>
@@ -20077,7 +20818,7 @@
         <v>452</v>
       </c>
       <c r="B19" t="s">
-        <v>1303</v>
+        <v>1340</v>
       </c>
       <c r="C19" t="s">
         <v>452</v>
@@ -20088,7 +20829,7 @@
         <v>452</v>
       </c>
       <c r="B20" t="s">
-        <v>1304</v>
+        <v>1341</v>
       </c>
       <c r="C20" t="s">
         <v>452</v>
@@ -20099,7 +20840,7 @@
         <v>452</v>
       </c>
       <c r="B21" t="s">
-        <v>1305</v>
+        <v>1342</v>
       </c>
       <c r="C21" t="s">
         <v>452</v>
@@ -20110,7 +20851,7 @@
         <v>452</v>
       </c>
       <c r="B22" t="s">
-        <v>1306</v>
+        <v>1343</v>
       </c>
       <c r="C22" t="s">
         <v>452</v>
@@ -20121,7 +20862,7 @@
         <v>452</v>
       </c>
       <c r="B23" t="s">
-        <v>1307</v>
+        <v>1344</v>
       </c>
       <c r="C23" t="s">
         <v>452</v>
@@ -20132,7 +20873,7 @@
         <v>452</v>
       </c>
       <c r="B24" t="s">
-        <v>1308</v>
+        <v>1345</v>
       </c>
       <c r="C24" t="s">
         <v>452</v>
@@ -20143,7 +20884,7 @@
         <v>452</v>
       </c>
       <c r="B25" t="s">
-        <v>1309</v>
+        <v>1346</v>
       </c>
       <c r="C25" t="s">
         <v>452</v>
@@ -20162,7 +20903,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>1310</v>
+        <v>1347</v>
       </c>
       <c r="B27" t="s">
         <v>452</v>
@@ -20176,10 +20917,10 @@
         <v>452</v>
       </c>
       <c r="B28" t="s">
-        <v>1311</v>
+        <v>1348</v>
       </c>
       <c r="C28" t="s">
-        <v>1312</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -20195,7 +20936,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>1313</v>
+        <v>1350</v>
       </c>
       <c r="B30" t="s">
         <v>452</v>
@@ -20209,7 +20950,7 @@
         <v>452</v>
       </c>
       <c r="B31" t="s">
-        <v>1314</v>
+        <v>1351</v>
       </c>
       <c r="C31" t="s">
         <v>452</v>
@@ -20220,7 +20961,7 @@
         <v>452</v>
       </c>
       <c r="B32" t="s">
-        <v>1315</v>
+        <v>1352</v>
       </c>
       <c r="C32" t="s">
         <v>452</v>
@@ -20231,7 +20972,7 @@
         <v>452</v>
       </c>
       <c r="B33" t="s">
-        <v>1316</v>
+        <v>1353</v>
       </c>
       <c r="C33" t="s">
         <v>452</v>
@@ -20250,7 +20991,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>1317</v>
+        <v>1354</v>
       </c>
       <c r="B35" t="s">
         <v>452</v>
@@ -20264,7 +21005,7 @@
         <v>452</v>
       </c>
       <c r="B36" t="s">
-        <v>1318</v>
+        <v>1355</v>
       </c>
       <c r="C36" t="s">
         <v>452</v>
@@ -20275,7 +21016,7 @@
         <v>452</v>
       </c>
       <c r="B37" t="s">
-        <v>1319</v>
+        <v>1356</v>
       </c>
       <c r="C37" t="s">
         <v>452</v>
@@ -20286,7 +21027,7 @@
         <v>452</v>
       </c>
       <c r="B38" t="s">
-        <v>1320</v>
+        <v>1357</v>
       </c>
       <c r="C38" t="s">
         <v>452</v>
@@ -20305,7 +21046,7 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>1321</v>
+        <v>1358</v>
       </c>
       <c r="B40" t="s">
         <v>452</v>

</xml_diff>

<commit_message>
refactor: đổi tên sản phẩm rõ ràng để dễ nhận biết Vỉ/Hộp/Vòi/Úp
- Bình RO-Vòi, Bình RO-Úp, Bình Kiềm-Vòi, Bình Kiềm-Úp, Vỉ 350ml, Hộp 350ml,
  Vỉ 500ml, Hộp 500ml — áp ở danh mục nền (catalog.sql) nên CSDL mới/khôi phục
  mặc định cũng dùng tên này.
- Cập nhật tên trong tệp nhập qaromi-nhap-T10.xlsx + script sinh tệp, các script
  migrate cũ và tài liệu API cho khớp.
- Đã nhập lại vào CSDL đang chạy (0 thêm mới / 572 cập nhật), 98/98 test pass.

Co-authored-by: CommandCodeBot <noreply@commandcode.ai>
</commit_message>
<xml_diff>
--- a/excel/qaromi-nhap-T10.xlsx
+++ b/excel/qaromi-nhap-T10.xlsx
@@ -123,7 +123,7 @@
     <t>Giám đốc</t>
   </si>
   <si>
-    <t>2026-10-06 14:16:45</t>
+    <t>2026-10-07 00:51:51</t>
   </si>
   <si>
     <t>NV002</t>
@@ -1515,7 +1515,7 @@
     <t>RO_19L_VOI</t>
   </si>
   <si>
-    <t>Nước Tinh Khiết RO QAROMI 19L (Bình Vòi)</t>
+    <t>Bình RO-Vòi</t>
   </si>
   <si>
     <t>Bình</t>
@@ -1533,7 +1533,7 @@
     <t>RO_19L_UP</t>
   </si>
   <si>
-    <t>Nước Tinh Khiết RO QAROMI 19L (Bình Úp)</t>
+    <t>Bình RO-Úp</t>
   </si>
   <si>
     <t>UP</t>
@@ -1542,19 +1542,19 @@
     <t>KIEM_19L_VOI</t>
   </si>
   <si>
-    <t>Nước Ion Kiềm QAROMI 19L (Bình Vòi)</t>
+    <t>Bình Kiềm-Vòi</t>
   </si>
   <si>
     <t>KIEM_19L_UP</t>
   </si>
   <si>
-    <t>Nước Ion Kiềm QAROMI 19L (Bình Úp)</t>
+    <t>Bình Kiềm-Úp</t>
   </si>
   <si>
     <t>VI_350ML</t>
   </si>
   <si>
-    <t>Nước Chai QAROMI 350ml (Vỉ)</t>
+    <t>Vỉ 350ml</t>
   </si>
   <si>
     <t>Vỉ</t>
@@ -1566,7 +1566,7 @@
     <t>HOP_350ML</t>
   </si>
   <si>
-    <t>Nước Chai QAROMI 350ml (Hộp)</t>
+    <t>Hộp 350ml</t>
   </si>
   <si>
     <t>Hộp</t>
@@ -1575,13 +1575,13 @@
     <t>VI_500ML</t>
   </si>
   <si>
-    <t>Nước Chai QAROMI 500ml (Vỉ)</t>
+    <t>Vỉ 500ml</t>
   </si>
   <si>
     <t>HOP_500ML</t>
   </si>
   <si>
-    <t>Nước Chai QAROMI 500ml (Hộp)</t>
+    <t>Hộp 500ml</t>
   </si>
   <si>
     <t>DV_BINH_NL</t>
@@ -4062,37 +4062,37 @@
     <t>TỒN ĐẦU KỲ 28/9/2026</t>
   </si>
   <si>
-    <t>KHO_HUE / Nước Ion Kiềm QAROMI 19L (Bình Vòi): 8</t>
-  </si>
-  <si>
-    <t>KHO_HUE / Nước Chai QAROMI 500ml (Vỉ): 192</t>
-  </si>
-  <si>
-    <t>KHO_HUE / Nước Chai QAROMI 350ml (Vỉ): 11</t>
-  </si>
-  <si>
-    <t>KHO_TANGAP / Nước Tinh Khiết RO QAROMI 19L (Bình Vòi): 1</t>
-  </si>
-  <si>
-    <t>KHO_TANGAP / Nước Ion Kiềm QAROMI 19L (Bình Vòi): 7</t>
-  </si>
-  <si>
-    <t>KHO_TANGAP / Nước Chai QAROMI 500ml (Vỉ): 214</t>
-  </si>
-  <si>
-    <t>KHO_TANGAP / Nước Chai QAROMI 350ml (Vỉ): 4</t>
-  </si>
-  <si>
-    <t>KHO_VP / Nước Ion Kiềm QAROMI 19L (Bình Vòi): 1</t>
-  </si>
-  <si>
-    <t>KHO_VP / Nước Chai QAROMI 500ml (Vỉ): 24</t>
-  </si>
-  <si>
-    <t>KHO_HALAM / Nước Chai QAROMI 500ml (Vỉ): 17</t>
-  </si>
-  <si>
-    <t>KHO_HALAM / Nước Chai QAROMI 350ml (Vỉ): 30</t>
+    <t>KHO_HUE / Bình Kiềm-Vòi: 8</t>
+  </si>
+  <si>
+    <t>KHO_HUE / Vỉ 500ml: 192</t>
+  </si>
+  <si>
+    <t>KHO_HUE / Vỉ 350ml: 11</t>
+  </si>
+  <si>
+    <t>KHO_TANGAP / Bình RO-Vòi: 1</t>
+  </si>
+  <si>
+    <t>KHO_TANGAP / Bình Kiềm-Vòi: 7</t>
+  </si>
+  <si>
+    <t>KHO_TANGAP / Vỉ 500ml: 214</t>
+  </si>
+  <si>
+    <t>KHO_TANGAP / Vỉ 350ml: 4</t>
+  </si>
+  <si>
+    <t>KHO_VP / Bình Kiềm-Vòi: 1</t>
+  </si>
+  <si>
+    <t>KHO_VP / Vỉ 500ml: 24</t>
+  </si>
+  <si>
+    <t>KHO_HALAM / Vỉ 500ml: 17</t>
+  </si>
+  <si>
+    <t>KHO_HALAM / Vỉ 350ml: 30</t>
   </si>
   <si>
     <t>KHO KHÔNG NHẬN RA (đã tạm xếp vào kho Tăng Áp)</t>

</xml_diff>